<commit_message>
Actualiza archivos filtrados automáticamente
</commit_message>
<xml_diff>
--- a/data/transformed/estadoObra_filtrado.xlsx
+++ b/data/transformed/estadoObra_filtrado.xlsx
@@ -419,12 +419,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Sucursal</t>
+          <t>sucursal</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Proyecto</t>
+          <t>proyecto</t>
         </is>
       </c>
     </row>

</xml_diff>